<commit_message>
The new changes integreted test cases in one spec file
</commit_message>
<xml_diff>
--- a/Admin/test-cases/Categories_Test_Cases.xlsx
+++ b/Admin/test-cases/Categories_Test_Cases.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G46"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -433,7 +433,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>TC_AP_292</v>
+        <v>TC_AP_678</v>
       </c>
       <c r="B2" t="str">
         <v>Categories</v>
@@ -458,7 +458,7 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>TC_AP_293</v>
+        <v>TC_AP_679</v>
       </c>
       <c r="B3" t="str">
         <v>Categories</v>
@@ -482,7 +482,7 @@
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>TC_AP_294</v>
+        <v>TC_AP_680</v>
       </c>
       <c r="B4" t="str">
         <v>Categories</v>
@@ -507,7 +507,7 @@
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>TC_AP_295</v>
+        <v>TC_AP_681</v>
       </c>
       <c r="B5" t="str">
         <v>Categories</v>
@@ -535,7 +535,7 @@
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>TC_AP_296</v>
+        <v>TC_AP_682</v>
       </c>
       <c r="B6" t="str">
         <v>Categories</v>
@@ -560,7 +560,7 @@
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>TC_AP_297</v>
+        <v>TC_AP_683</v>
       </c>
       <c r="B7" t="str">
         <v>Categories</v>
@@ -584,7 +584,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TC_AP_298</v>
+        <v>TC_AP_684</v>
       </c>
       <c r="B8" t="str">
         <v>Categories</v>
@@ -607,7 +607,7 @@
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
-        <v>TC_AP_299</v>
+        <v>TC_AP_685</v>
       </c>
       <c r="B9" t="str">
         <v>Categories</v>
@@ -631,7 +631,7 @@
     </row>
     <row r="10" xml:space="preserve">
       <c r="A10" t="str">
-        <v>TC_AP_300</v>
+        <v>TC_AP_686</v>
       </c>
       <c r="B10" t="str">
         <v>Categories</v>
@@ -656,7 +656,7 @@
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str">
-        <v>TC_AP_301</v>
+        <v>TC_AP_687</v>
       </c>
       <c r="B11" t="str">
         <v>Categories</v>
@@ -680,7 +680,7 @@
     </row>
     <row r="12" xml:space="preserve">
       <c r="A12" t="str">
-        <v>TC_AP_302</v>
+        <v>TC_AP_688</v>
       </c>
       <c r="B12" t="str">
         <v>Categories</v>
@@ -704,7 +704,7 @@
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str">
-        <v>TC_AP_303</v>
+        <v>TC_AP_689</v>
       </c>
       <c r="B13" t="str">
         <v>Categories</v>
@@ -728,7 +728,7 @@
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str">
-        <v>TC_AP_304</v>
+        <v>TC_AP_690</v>
       </c>
       <c r="B14" t="str">
         <v>Categories</v>
@@ -752,24 +752,25 @@
     </row>
     <row r="15" xml:space="preserve">
       <c r="A15" t="str">
-        <v>TC_AP_305</v>
+        <v>TC_AP_691</v>
       </c>
       <c r="B15" t="str">
         <v>Categories</v>
       </c>
       <c r="C15" t="str">
-        <v>Verify category can be edited</v>
+        <v>Verify category name and description can be edited from the edit form</v>
       </c>
       <c r="D15" t="str">
-        <v>An existing category is available in the list.</v>
+        <v>A category exists in the list with no assigned groups.</v>
       </c>
       <c r="E15" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Click the Edit icon for a category.
-• Update the category name and/or description.
-• Save the changes.</v>
+        <v xml:space="preserve">• Click the Edit (pencil) icon for the category row.
+• Verify the edit form shows Category Name, Assigned Groups, Description, Update, Cancel, and Back.
+• Update the category name and description.
+• Click the "Update" button.</v>
       </c>
       <c r="F15" t="str">
-        <v>Category is updated successfully and the list reflects the new values.</v>
+        <v>Category is updated successfully. The Categories list shows the new name and description.</v>
       </c>
       <c r="G15" t="str">
         <v/>
@@ -777,47 +778,49 @@
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str">
-        <v>TC_AP_306</v>
+        <v>TC_AP_692</v>
       </c>
       <c r="B16" t="str">
         <v>Categories</v>
       </c>
       <c r="C16" t="str">
-        <v>Verify assigned groups can be updated on edit category</v>
+        <v>Verify assigned groups can be added on the edit category form</v>
       </c>
       <c r="D16" t="str">
-        <v>An existing category is available for editing.</v>
+        <v>A category with zero assigned groups exists and groups are available in the system.</v>
       </c>
       <c r="E16" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Open Edit for a category.
-• Add or remove assigned groups.
-• Save the changes.</v>
+        <v xml:space="preserve">• Click Edit for the category.
+• Open Assigned Groups, search for a group, select it, and click Add.
+• Click the "Update" button.</v>
       </c>
       <c r="F16" t="str">
-        <v>Assigned groups are updated and Assigned Groups count changes accordingly.</v>
+        <v>Assigned groups are saved and the Assigned Groups count increases in the list.</v>
       </c>
       <c r="G16" t="str">
         <v/>
       </c>
     </row>
-    <row r="17">
+    <row r="17" xml:space="preserve">
       <c r="A17" t="str">
-        <v>TC_AP_307</v>
+        <v>TC_AP_693</v>
       </c>
       <c r="B17" t="str">
         <v>Categories</v>
       </c>
       <c r="C17" t="str">
-        <v>Verify delete category shows confirmation modal</v>
+        <v>Verify delete category shows confirmation modal with Yes and Cancel</v>
       </c>
       <c r="D17" t="str">
-        <v>An existing category is available in the list.</v>
-      </c>
-      <c r="E17" t="str">
-        <v>• Click the Delete icon for a category.</v>
+        <v>A deletable category (no assigned groups) exists in the list.</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click the Delete (trash) icon for the category row.
+• Observe the confirmation dialog.
+• Click "Cancel".</v>
       </c>
       <c r="F17" t="str">
-        <v>A confirmation dialog appears asking to confirm category deletion.</v>
+        <v>Modal displays "Are you sure you want to delete this category?" with Yes and Cancel. Category remains after Cancel.</v>
       </c>
       <c r="G17" t="str">
         <v/>
@@ -825,20 +828,20 @@
     </row>
     <row r="18" xml:space="preserve">
       <c r="A18" t="str">
-        <v>TC_AP_308</v>
+        <v>TC_AP_694</v>
       </c>
       <c r="B18" t="str">
         <v>Categories</v>
       </c>
       <c r="C18" t="str">
-        <v>Verify category can be deleted successfully</v>
+        <v>Verify category with no assigned groups can be deleted successfully</v>
       </c>
       <c r="D18" t="str">
-        <v>A deletable test category exists with no blocking dependencies.</v>
+        <v>A test category exists with zero assigned groups.</v>
       </c>
       <c r="E18" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Click Delete for the test category.
-• Confirm deletion in the modal.</v>
+        <v xml:space="preserve">• Click Delete for the category.
+• Click "Yes" on the confirmation modal.</v>
       </c>
       <c r="F18" t="str">
         <v>Category is deleted and no longer appears in the Categories list.</v>
@@ -849,178 +852,694 @@
     </row>
     <row r="19" xml:space="preserve">
       <c r="A19" t="str">
-        <v>TC_AP_309</v>
+        <v>TC_AP_702</v>
       </c>
       <c r="B19" t="str">
         <v>Categories</v>
       </c>
       <c r="C19" t="str">
+        <v>Verify delete is blocked when category has assigned groups</v>
+      </c>
+      <c r="D19" t="str">
+        <v>A category with one or more assigned groups exists in the list.</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Delete for a category that has assigned groups.
+• Read the warning message.
+• Click "OK" to dismiss the modal.</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Delete Group modal appears: "Category cannot be deleted while groups are assigned. Please remove all assigned groups first." Category is not deleted.</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC_AP_695</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C20" t="str">
         <v>Verify pagination on categories list</v>
       </c>
-      <c r="D19" t="str">
+      <c r="D20" t="str">
         <v>More categories exist than fit on one page.</v>
       </c>
-      <c r="E19" t="str" xml:space="preserve">
+      <c r="E20" t="str" xml:space="preserve">
         <v xml:space="preserve">• Navigate to Categories list.
 • Use Next/Previous or page number controls.</v>
       </c>
-      <c r="F19" t="str">
+      <c r="F20" t="str">
         <v>Pagination navigates between pages and displays correct item range.</v>
       </c>
-      <c r="G19" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str">
-        <v>TC_AP_310</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C20" t="str">
+      <c r="G20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC_AP_696</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C21" t="str">
         <v>Verify sort by Name ascending and descending</v>
       </c>
-      <c r="D20" t="str">
+      <c r="D21" t="str">
         <v>Multiple categories exist in the list.</v>
       </c>
-      <c r="E20" t="str" xml:space="preserve">
+      <c r="E21" t="str" xml:space="preserve">
         <v xml:space="preserve">• Click Sort Ascending on the Name column.
 • Observe the order.
 • Click Sort Descending on the Name column.</v>
       </c>
-      <c r="F20" t="str">
+      <c r="F21" t="str">
         <v>Categories are sorted alphabetically by name in ascending and descending order.</v>
       </c>
-      <c r="G20" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str">
-        <v>TC_AP_311</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C21" t="str">
+      <c r="G21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC_AP_697</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C22" t="str">
         <v>Verify sort by Created On column</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D22" t="str">
         <v>Multiple categories exist with different created dates.</v>
       </c>
-      <c r="E21" t="str" xml:space="preserve">
+      <c r="E22" t="str" xml:space="preserve">
         <v xml:space="preserve">• Sort by Created On ascending.
 • Sort by Created On descending.</v>
       </c>
-      <c r="F21" t="str">
+      <c r="F22" t="str">
         <v>Categories are ordered by Created On date correctly in both directions.</v>
       </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22" xml:space="preserve">
-      <c r="A22" t="str">
-        <v>TC_AP_312</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C22" t="str">
+      <c r="G22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC_AP_698</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C23" t="str">
         <v>Verify sort by Updated On column</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D23" t="str">
         <v>Multiple categories exist with different updated dates.</v>
       </c>
-      <c r="E22" t="str" xml:space="preserve">
+      <c r="E23" t="str" xml:space="preserve">
         <v xml:space="preserve">• Sort by Updated On ascending.
 • Sort by Updated On descending.</v>
       </c>
-      <c r="F22" t="str">
+      <c r="F23" t="str">
         <v>Categories are ordered by Updated On date correctly in both directions.</v>
       </c>
-      <c r="G22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23" xml:space="preserve">
-      <c r="A23" t="str">
-        <v>TC_AP_313</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C23" t="str">
+      <c r="G23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC_AP_699</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C24" t="str">
         <v>Verify categories list data matches the category list API</v>
       </c>
-      <c r="D23" t="str">
+      <c r="D24" t="str">
         <v>User is logged in and Categories API is accessible.</v>
       </c>
-      <c r="E23" t="str" xml:space="preserve">
+      <c r="E24" t="str" xml:space="preserve">
         <v xml:space="preserve">• Load the Categories page.
 • Compare visible category names with GET /category?page=0&amp;size=25&amp;search=&amp;sort=createdAt,desc response.</v>
       </c>
-      <c r="F23" t="str">
+      <c r="F24" t="str">
         <v>UI list data is consistent with the category list API response.</v>
       </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="24" xml:space="preserve">
-      <c r="A24" t="str">
-        <v>TC_AP_314</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C24" t="str">
+      <c r="G24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC_AP_700</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C25" t="str">
         <v>Verify Description field is optional on create category</v>
       </c>
-      <c r="D24" t="str">
+      <c r="D25" t="str">
         <v>User is on the Create Category page.</v>
       </c>
-      <c r="E24" t="str" xml:space="preserve">
+      <c r="E25" t="str" xml:space="preserve">
         <v xml:space="preserve">• Enter only a valid Category Name.
 • Leave Description empty.
 • Click Create.</v>
       </c>
-      <c r="F24" t="str">
+      <c r="F25" t="str">
         <v>Category is created successfully without a description.</v>
       </c>
-      <c r="G24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
-      <c r="A25" t="str">
-        <v>TC_AP_315</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Categories</v>
-      </c>
-      <c r="C25" t="str">
+      <c r="G25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC_AP_701</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C26" t="str">
         <v>Verify category name trims leading and trailing spaces</v>
       </c>
-      <c r="D25" t="str">
+      <c r="D26" t="str">
         <v>User is on the Create Category page.</v>
       </c>
-      <c r="E25" t="str" xml:space="preserve">
+      <c r="E26" t="str" xml:space="preserve">
         <v xml:space="preserve">• Enter a category name with leading and trailing spaces.
 • Click Create.
 • Check the saved name in the list.</v>
       </c>
-      <c r="F25" t="str">
+      <c r="F26" t="str">
         <v>Category is saved with trimmed name (no leading/trailing spaces).</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC_AP_703</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Negative - Verify duplicate category name is not allowed on create</v>
+      </c>
+      <c r="D27" t="str">
+        <v>A category with a known name already exists in the system.</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Create Category.
+• Enter the same category name as an existing category.
+• Enter description and click Create.</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Category is not created. An error message indicates the name must be unique.</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>TC_AP_704</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Negative - Verify category cannot be created with blank or whitespace-only name</v>
+      </c>
+      <c r="D28" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter only spaces in the Category Name field.
+• Click Create.</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Validation error is shown and category is not created.</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>TC_AP_705</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Negative - Verify category name rejects special characters on create</v>
+      </c>
+      <c r="D29" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter a category name containing special characters (e.g. Test@#$Category).
+• Click Create.</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Validation error is shown and category is not created.</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>TC_AP_706</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Negative - Verify category cannot be updated with an empty name</v>
+      </c>
+      <c r="D30" t="str">
+        <v>An existing category is available for editing.</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Edit for the category.
+• Clear the Category Name field completely.
+• Click Update.</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Validation error is shown for Category Name and changes are not saved.</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>TC_AP_707</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Negative - Verify duplicate category name is not allowed on edit</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Two distinct categories exist in the list (Category A and Category B).</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Edit for Category B.
+• Change the name to match Category A exactly.
+• Click Update.</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Update is rejected with a duplicate-name error. Category B retains its original name.</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>TC_AP_708</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Negative - Verify delete is not performed when confirmation modal is cancelled</v>
+      </c>
+      <c r="D32" t="str">
+        <v>A deletable category (zero assigned groups) exists.</v>
+      </c>
+      <c r="E32" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Delete for the category.
+• On the confirmation modal, click Cancel.
+• Search for the category in the list.</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Modal closes and the category still exists in the Categories list.</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>TC_AP_709</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Negative - Verify search with only spaces does not break the list</v>
+      </c>
+      <c r="D33" t="str">
+        <v>User is on the Categories list page with data loaded.</v>
+      </c>
+      <c r="E33" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter only spaces in the Search field.
+• Press Enter or trigger search.</v>
+      </c>
+      <c r="F33" t="str">
+        <v>No error occurs. List either shows all categories or treats input as empty search.</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>TC_AP_710</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Edge - Verify closing Assigned Groups dropdown without Add does not assign groups</v>
+      </c>
+      <c r="D34" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E34" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Open Assigned Groups dropdown and search for a group.
+• Select a checkbox but do not click Add, or close the dropdown without adding.
+• Enter a valid category name and click Create.</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Category is created only with groups explicitly added via Add. Unconfirmed selections are not saved.</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>TC_AP_711</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Edge - Verify Cancel on edit discards unsaved changes</v>
+      </c>
+      <c r="D35" t="str">
+        <v>An existing category is open on the edit form.</v>
+      </c>
+      <c r="E35" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Change the category name and description.
+• Click Cancel without clicking Update.
+• Locate the original category in the list.</v>
+      </c>
+      <c r="F35" t="str">
+        <v>User returns to the list. Original name and description are unchanged.</v>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>TC_AP_712</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Edge - Verify Back link on edit returns to list without saving changes</v>
+      </c>
+      <c r="D36" t="str">
+        <v>An existing category is open on the edit form.</v>
+      </c>
+      <c r="E36" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Modify the category name.
+• Click the Back link.
+• Verify the category in the list.</v>
+      </c>
+      <c r="F36" t="str">
+        <v>User is navigated to Categories list. Unsaved edits are not applied.</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>TC_AP_713</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Edge - Verify edit form is pre-populated with existing category data</v>
+      </c>
+      <c r="D37" t="str">
+        <v>A category with name, description, and assigned groups exists.</v>
+      </c>
+      <c r="E37" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Edit for the category.
+• Observe Category Name, Description, and Assigned Groups fields.</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Form shows the current category name, description, and already-assigned group tags.</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>TC_AP_714</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Edge - Verify assigned group can be removed from edit form using tag remove icon</v>
+      </c>
+      <c r="D38" t="str">
+        <v>A category with at least one assigned group exists.</v>
+      </c>
+      <c r="E38" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Edit for the category.
+• Click the remove (x) icon on an assigned group tag.
+• Click Update.</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Group is removed from the category. Assigned Groups count decreases in the list.</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>TC_AP_715</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Edge - Verify category name with maximum allowed length</v>
+      </c>
+      <c r="D39" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E39" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter a category name at the maximum permitted character length.
+• Click Create.</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Category is created successfully when name is within the allowed limit.</v>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>TC_AP_716</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Edge - Verify category name exceeding maximum length is rejected</v>
+      </c>
+      <c r="D40" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E40" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter a category name longer than the maximum permitted length.
+• Click Create.</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Validation error is shown or input is truncated. Category is not saved with invalid length.</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>TC_AP_717</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Edge - Verify very long description is accepted or validated on create</v>
+      </c>
+      <c r="D41" t="str">
+        <v>User is on the Create Category page.</v>
+      </c>
+      <c r="E41" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter a valid category name.
+• Paste a very long description (multi-paragraph text).
+• Click Create.</v>
+      </c>
+      <c r="F41" t="str">
+        <v>System either accepts the description within limits or shows a validation message.</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>TC_AP_718</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Edge - Verify Assigned Groups search with no matching group shows empty state</v>
+      </c>
+      <c r="D42" t="str">
+        <v>User is on Create or Edit Category form.</v>
+      </c>
+      <c r="E42" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Open Assigned Groups dropdown.
+• Search for a random string that matches no group.</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Dropdown shows no matching groups or an empty-state message.</v>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>TC_AP_719</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Edge - Verify pagination controls are disabled on a single-page list</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Total categories fit on one page (e.g. fewer than page size).</v>
+      </c>
+      <c r="E43" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Open the Categories list.
+• Observe Previous, Next, and page number controls.</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Pagination shows "1-N of N items". Previous and Next controls are disabled.</v>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>TC_AP_720</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Edge - Verify rapid double-click on Create does not create duplicate categories</v>
+      </c>
+      <c r="D44" t="str">
+        <v>User is on the Create Category page with valid data entered.</v>
+      </c>
+      <c r="E44" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Enter a unique category name and description.
+• Double-click the Create button quickly.
+• Search for the category name.</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Only one category with that name is created.</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>TC_AP_721</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Edge - Verify rapid double-click on Update does not cause duplicate updates or errors</v>
+      </c>
+      <c r="D45" t="str">
+        <v>User is on the edit form for an existing category.</v>
+      </c>
+      <c r="E45" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Change the description.
+• Double-click the Update button quickly.</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Category is updated once without duplicate API errors or inconsistent list data.</v>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>TC_AP_722</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Categories</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Edge - Verify delete blocked modal dismisses with OK and category remains</v>
+      </c>
+      <c r="D46" t="str">
+        <v>A category with assigned groups exists.</v>
+      </c>
+      <c r="E46" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Click Delete for the category.
+• On the blocked-delete modal, click OK.
+• Verify the category is still in the list.</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Modal closes. Category is not deleted and Assigned Groups count is unchanged.</v>
+      </c>
+      <c r="G46" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>